<commit_message>
fix(web): replace deprecated apple-mobile-web-app-capable meta tag and handle wasm unreachable errors in SQLite recovery
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tmp/20260316-collection.xlsx
+++ b/docs/tmp/20260316-collection.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\ai\recycling\docs\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63BD7600-E493-4E0C-B9E6-B953081F84DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DEB774-F211-487D-AAE4-385FD30EFE95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -491,7 +491,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -501,6 +501,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -517,7 +523,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -531,6 +537,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -802,7 +811,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>46097</v>
       </c>
@@ -834,7 +843,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>15</v>
@@ -843,7 +852,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
         <v>17</v>
@@ -852,28 +861,28 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="1:12" s="10" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="9">
         <v>39.6</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="9">
         <v>3.3</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="9">
         <v>39.6</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
@@ -901,7 +910,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
         <v>24</v>
@@ -943,7 +952,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" s="7" customFormat="1" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A9" s="6"/>
       <c r="B9" s="6" t="s">
         <v>28</v>
@@ -967,7 +976,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A10" s="5"/>
       <c r="B10" s="5" t="s">
         <v>32</v>
@@ -993,7 +1002,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
         <v>34</v>
@@ -1018,7 +1027,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
         <v>37</v>
@@ -1044,7 +1053,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
         <v>40</v>
@@ -1070,7 +1079,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
         <v>43</v>
@@ -1098,7 +1107,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
         <v>46</v>
@@ -1184,7 +1193,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
         <v>55</v>
@@ -1193,7 +1202,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
         <v>57</v>
@@ -1202,7 +1211,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
         <v>58</v>
@@ -1228,7 +1237,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
         <v>61</v>
@@ -1246,7 +1255,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
         <v>64</v>
@@ -1274,7 +1283,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="5" t="s">
         <v>67</v>
@@ -1297,7 +1306,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
         <v>69</v>
@@ -1323,7 +1332,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="5" t="s">
         <v>72</v>
@@ -1346,7 +1355,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
@@ -1357,7 +1366,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="5" t="s">
         <v>74</v>
@@ -1380,7 +1389,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
       <c r="B29" s="5" t="s">
         <v>77</v>
@@ -1403,7 +1412,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="5" t="s">
         <v>80</v>
@@ -1429,7 +1438,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="5" t="s">
         <v>82</v>
@@ -1449,7 +1458,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
         <v>84</v>
@@ -1475,7 +1484,7 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
         <v>87</v>

</xml_diff>